<commit_message>
docs: add By Job Title summary tab + PDF export to coding disclosure
Workbook now has a fifth tab 'By Job Title' (actions/hours/value rolled up per skillset via COUNTIF/SUMIF). Adds JHI_Coding_Disclosure.pdf, a print/share-ready 3-page PDF rendered from the same source data (reportlab) so xlsx and PDF stay in sync. Updates generator + README; reportlab added as tooling-only dependency for regeneration.

Co-authored-by: marcellmiller27 <marcellmiller27@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/disclosure/JHI_Coding_Disclosure.xlsx
+++ b/docs/disclosure/JHI_Coding_Disclosure.xlsx
@@ -10,7 +10,8 @@
     <sheet name="Disclosure" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Rate Card" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Subsystem Summary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Notes &amp; Disclosure" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="By Job Title" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Notes &amp; Disclosure" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2986,6 +2987,301 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Summary by Job Title (skillset)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Job title (skillset)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Actions</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Est. hours</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Value ($)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Mid rate ($/hr)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Backend Engineer</t>
+        </is>
+      </c>
+      <c r="B4" s="8">
+        <f>COUNTIF(Disclosure!$C$5:$C$48,A4)</f>
+        <v/>
+      </c>
+      <c r="C4" s="8">
+        <f>SUMIF(Disclosure!$C$5:$C$48,A4,Disclosure!$F$5:$F$48)</f>
+        <v/>
+      </c>
+      <c r="D4" s="9">
+        <f>SUMIF(Disclosure!$C$5:$C$48,A4,Disclosure!$G$5:$G$48)</f>
+        <v/>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Security Engineer</t>
+        </is>
+      </c>
+      <c r="B5" s="8">
+        <f>COUNTIF(Disclosure!$C$5:$C$48,A5)</f>
+        <v/>
+      </c>
+      <c r="C5" s="8">
+        <f>SUMIF(Disclosure!$C$5:$C$48,A5,Disclosure!$F$5:$F$48)</f>
+        <v/>
+      </c>
+      <c r="D5" s="9">
+        <f>SUMIF(Disclosure!$C$5:$C$48,A5,Disclosure!$G$5:$G$48)</f>
+        <v/>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Frontend Engineer</t>
+        </is>
+      </c>
+      <c r="B6" s="8">
+        <f>COUNTIF(Disclosure!$C$5:$C$48,A6)</f>
+        <v/>
+      </c>
+      <c r="C6" s="8">
+        <f>SUMIF(Disclosure!$C$5:$C$48,A6,Disclosure!$F$5:$F$48)</f>
+        <v/>
+      </c>
+      <c r="D6" s="9">
+        <f>SUMIF(Disclosure!$C$5:$C$48,A6,Disclosure!$G$5:$G$48)</f>
+        <v/>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Integration Engineer</t>
+        </is>
+      </c>
+      <c r="B7" s="8">
+        <f>COUNTIF(Disclosure!$C$5:$C$48,A7)</f>
+        <v/>
+      </c>
+      <c r="C7" s="8">
+        <f>SUMIF(Disclosure!$C$5:$C$48,A7,Disclosure!$F$5:$F$48)</f>
+        <v/>
+      </c>
+      <c r="D7" s="9">
+        <f>SUMIF(Disclosure!$C$5:$C$48,A7,Disclosure!$G$5:$G$48)</f>
+        <v/>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Data Scientist / Quant</t>
+        </is>
+      </c>
+      <c r="B8" s="8">
+        <f>COUNTIF(Disclosure!$C$5:$C$48,A8)</f>
+        <v/>
+      </c>
+      <c r="C8" s="8">
+        <f>SUMIF(Disclosure!$C$5:$C$48,A8,Disclosure!$F$5:$F$48)</f>
+        <v/>
+      </c>
+      <c r="D8" s="9">
+        <f>SUMIF(Disclosure!$C$5:$C$48,A8,Disclosure!$G$5:$G$48)</f>
+        <v/>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="B9" s="8">
+        <f>COUNTIF(Disclosure!$C$5:$C$48,A9)</f>
+        <v/>
+      </c>
+      <c r="C9" s="8">
+        <f>SUMIF(Disclosure!$C$5:$C$48,A9,Disclosure!$F$5:$F$48)</f>
+        <v/>
+      </c>
+      <c r="D9" s="9">
+        <f>SUMIF(Disclosure!$C$5:$C$48,A9,Disclosure!$G$5:$G$48)</f>
+        <v/>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>UX / UI Designer</t>
+        </is>
+      </c>
+      <c r="B10" s="8">
+        <f>COUNTIF(Disclosure!$C$5:$C$48,A10)</f>
+        <v/>
+      </c>
+      <c r="C10" s="8">
+        <f>SUMIF(Disclosure!$C$5:$C$48,A10,Disclosure!$F$5:$F$48)</f>
+        <v/>
+      </c>
+      <c r="D10" s="9">
+        <f>SUMIF(Disclosure!$C$5:$C$48,A10,Disclosure!$G$5:$G$48)</f>
+        <v/>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>QA Engineer</t>
+        </is>
+      </c>
+      <c r="B11" s="8">
+        <f>COUNTIF(Disclosure!$C$5:$C$48,A11)</f>
+        <v/>
+      </c>
+      <c r="C11" s="8">
+        <f>SUMIF(Disclosure!$C$5:$C$48,A11,Disclosure!$F$5:$F$48)</f>
+        <v/>
+      </c>
+      <c r="D11" s="9">
+        <f>SUMIF(Disclosure!$C$5:$C$48,A11,Disclosure!$G$5:$G$48)</f>
+        <v/>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>DevOps / Cloud Engineer</t>
+        </is>
+      </c>
+      <c r="B12" s="8">
+        <f>COUNTIF(Disclosure!$C$5:$C$48,A12)</f>
+        <v/>
+      </c>
+      <c r="C12" s="8">
+        <f>SUMIF(Disclosure!$C$5:$C$48,A12,Disclosure!$F$5:$F$48)</f>
+        <v/>
+      </c>
+      <c r="D12" s="9">
+        <f>SUMIF(Disclosure!$C$5:$C$48,A12,Disclosure!$G$5:$G$48)</f>
+        <v/>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Tech Lead / Architect</t>
+        </is>
+      </c>
+      <c r="B13" s="8">
+        <f>COUNTIF(Disclosure!$C$5:$C$48,A13)</f>
+        <v/>
+      </c>
+      <c r="C13" s="8">
+        <f>SUMIF(Disclosure!$C$5:$C$48,A13,Disclosure!$F$5:$F$48)</f>
+        <v/>
+      </c>
+      <c r="D13" s="9">
+        <f>SUMIF(Disclosure!$C$5:$C$48,A13,Disclosure!$G$5:$G$48)</f>
+        <v/>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B14" s="6">
+        <f>SUM(B4:B13)</f>
+        <v/>
+      </c>
+      <c r="C14" s="6">
+        <f>SUM(C4:C13)</f>
+        <v/>
+      </c>
+      <c r="D14" s="7">
+        <f>SUM(D4:D13)</f>
+        <v/>
+      </c>
+      <c r="E14" s="6" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>